<commit_message>
Atualização no arquivo de Tasks da Sprint 3
</commit_message>
<xml_diff>
--- a/DOCS/sprints/sprint-03/TasksSprint3.xlsx
+++ b/DOCS/sprints/sprint-03/TasksSprint3.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>Backlog</t>
   </si>
@@ -60,7 +60,7 @@
     <t>William</t>
   </si>
   <si>
-    <t xml:space="preserve">Para Fazer</t>
+    <t xml:space="preserve">Em Andamento</t>
   </si>
   <si>
     <t xml:space="preserve">Cadastrar, editar e remover documentos,metadados, preservando o vínculo entre evidência e resposta final.</t>
@@ -166,9 +166,6 @@
   </si>
   <si>
     <t xml:space="preserve">Implementar feedback visual de carregamento (Skeleton ou Spinner) e mensagens de erro amigáveis se nada for encontrado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Em Andamento</t>
   </si>
   <si>
     <t xml:space="preserve">Permitir consulta direta, localizar respostas cadastradas quando houver aderência e orientar o usuário quando a busca não resolver o caso.</t>
@@ -428,7 +425,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="15">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -469,7 +466,6 @@
     </font>
     <font>
       <sz val="14.000000"/>
-      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -511,11 +507,6 @@
     </font>
     <font>
       <sz val="14.000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="14.000000"/>
-      <color indexed="64"/>
       <name val="Times New Roman"/>
     </font>
     <font>
@@ -546,6 +537,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFE597"/>
+        <bgColor rgb="FFFFE597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE5E7EB"/>
         <bgColor rgb="FFE5E7EB"/>
       </patternFill>
@@ -560,12 +557,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="0"/>
         <bgColor theme="0" tint="0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE597"/>
-        <bgColor rgb="FFFFE597"/>
       </patternFill>
     </fill>
     <fill>
@@ -659,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="47">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -694,25 +685,25 @@
     <xf fontId="1" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="9" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="9" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="10" fillId="5" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="10" fillId="6" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="10" fillId="5" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="10" fillId="6" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="10" fillId="5" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="10" fillId="6" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="11" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -721,7 +712,7 @@
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="12" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="12" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -730,7 +721,7 @@
     <xf fontId="7" fillId="0" borderId="1" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="8" fillId="6" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="8" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -742,7 +733,7 @@
     <xf fontId="7" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="13" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="6" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -751,22 +742,10 @@
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="6" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="1" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="7" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="8" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="2" fillId="4" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="2" fillId="5" borderId="1" numFmtId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -784,19 +763,13 @@
     <xf fontId="1" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="6" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="6" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="8" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="14" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="1" fillId="7" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="14" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="13" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -805,22 +778,16 @@
     <xf fontId="10" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="15" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="14" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1195,6 +1162,15 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
+        <c:dLbls>
+          <c:showBubbleSize val="0"/>
+          <c:showCatName val="0"/>
+          <c:showLeaderLines val="0"/>
+          <c:showLegendKey val="0"/>
+          <c:showPercent val="0"/>
+          <c:showSerName val="0"/>
+          <c:showVal val="0"/>
+        </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
         <c:axId val="2140841477"/>
@@ -2702,7 +2678,7 @@
         <v>46170</v>
       </c>
       <c r="L5" s="22">
-        <f>SUM(L4-28.583)</f>
+        <f t="shared" ref="L5:L10" si="0">SUM(L4-28.583)</f>
         <v>314.41700000000003</v>
       </c>
       <c r="M5" s="20">
@@ -2740,7 +2716,7 @@
         <v>46171</v>
       </c>
       <c r="L6" s="23">
-        <f>SUM(L5-28.583)</f>
+        <f t="shared" si="0"/>
         <v>285.83400000000006</v>
       </c>
       <c r="M6" s="20">
@@ -2762,7 +2738,7 @@
         <v>46172</v>
       </c>
       <c r="L7" s="23">
-        <f>SUM(L6-28.583)</f>
+        <f t="shared" si="0"/>
         <v>257.25100000000009</v>
       </c>
       <c r="M7" s="27">
@@ -2800,7 +2776,7 @@
         <v>46173</v>
       </c>
       <c r="L8" s="23">
-        <f>SUM(L7-28.583)</f>
+        <f t="shared" si="0"/>
         <v>228.66800000000009</v>
       </c>
       <c r="M8" s="20">
@@ -2837,7 +2813,7 @@
         <v>46174</v>
       </c>
       <c r="L9" s="23">
-        <f>SUM(L8-28.583)</f>
+        <f t="shared" si="0"/>
         <v>200.08500000000009</v>
       </c>
       <c r="M9" s="20">
@@ -2860,7 +2836,7 @@
       <c r="E10" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F10" s="18" t="s">
+      <c r="F10" s="10" t="s">
         <v>14</v>
       </c>
       <c r="G10" s="8" t="s">
@@ -2874,7 +2850,7 @@
         <v>46175</v>
       </c>
       <c r="L10" s="23">
-        <f>SUM(L9-28.583)</f>
+        <f t="shared" si="0"/>
         <v>171.50200000000009</v>
       </c>
       <c r="M10" s="20">
@@ -2895,7 +2871,7 @@
         <v>46176</v>
       </c>
       <c r="L11" s="23">
-        <f>SUM(L10-28.583)</f>
+        <f t="shared" ref="L11:L15" si="1">SUM(L10-28.583)</f>
         <v>142.9190000000001</v>
       </c>
       <c r="M11" s="20">
@@ -2903,28 +2879,28 @@
       </c>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="31" t="s">
+      <c r="A12" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="32" t="s">
+      <c r="E12" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="F12" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G12" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="H12" s="32">
+      <c r="H12" s="11">
         <v>17</v>
       </c>
       <c r="I12" s="18"/>
@@ -2932,7 +2908,7 @@
         <v>46177</v>
       </c>
       <c r="L12" s="23">
-        <f>SUM(L11-28.583)</f>
+        <f t="shared" si="1"/>
         <v>114.3360000000001</v>
       </c>
       <c r="M12" s="20">
@@ -2940,28 +2916,28 @@
       </c>
     </row>
     <row r="13" ht="19.5" customHeight="1">
-      <c r="A13" s="31" t="s">
+      <c r="A13" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="D13" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="E13" s="34" t="s">
+      <c r="E13" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="33" t="s">
+      <c r="F13" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="31" t="s">
-        <v>51</v>
-      </c>
-      <c r="H13" s="32">
+      <c r="H13" s="11">
         <v>17</v>
       </c>
       <c r="I13" s="18"/>
@@ -2969,7 +2945,7 @@
         <v>46178</v>
       </c>
       <c r="L13" s="23">
-        <f>SUM(L12-28.583)</f>
+        <f t="shared" si="1"/>
         <v>85.7530000000001</v>
       </c>
       <c r="M13" s="20">
@@ -2990,7 +2966,7 @@
         <v>46179</v>
       </c>
       <c r="L14" s="23">
-        <f>SUM(L13-28.583)</f>
+        <f t="shared" si="1"/>
         <v>57.170000000000101</v>
       </c>
       <c r="M14" s="20">
@@ -2998,28 +2974,28 @@
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
-      <c r="A15" s="31" t="s">
+      <c r="A15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="C15" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="D15" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="E15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="E15" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="33" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="H15" s="32">
+      <c r="H15" s="11">
         <v>21</v>
       </c>
       <c r="I15" s="18"/>
@@ -3027,7 +3003,7 @@
         <v>46180</v>
       </c>
       <c r="L15" s="23">
-        <f>SUM(L14-28.583)</f>
+        <f t="shared" si="1"/>
         <v>28.587000000000103</v>
       </c>
       <c r="M15" s="20">
@@ -3055,98 +3031,96 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="C17" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="31" t="s">
+      <c r="D17" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="D17" s="31" t="s">
+      <c r="E17" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="34" t="s">
+      <c r="F17" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="F17" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G17" s="31" t="s">
+      <c r="H17" s="11">
+        <v>11</v>
+      </c>
+      <c r="I17" s="32"/>
+      <c r="K17" s="33"/>
+      <c r="L17" s="33"/>
+      <c r="M17" s="33"/>
+    </row>
+    <row r="18" ht="19.5" customHeight="1">
+      <c r="A18" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="H17" s="32">
+      <c r="C18" s="34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>68</v>
+      </c>
+      <c r="F18" s="36" t="s">
+        <v>69</v>
+      </c>
+      <c r="G18" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="H18" s="37">
         <v>11</v>
       </c>
-      <c r="I17" s="36">
-        <v>46181</v>
-      </c>
-      <c r="K17" s="37"/>
-      <c r="L17" s="37"/>
-      <c r="M17" s="37"/>
-    </row>
-    <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="E18" s="39" t="s">
+      <c r="I18" s="32">
+        <v>46179</v>
+      </c>
+      <c r="K18" s="33"/>
+      <c r="L18" s="33"/>
+      <c r="M18" s="33"/>
+    </row>
+    <row r="19" ht="37.5">
+      <c r="A19" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" s="36" t="s">
         <v>69</v>
       </c>
-      <c r="F18" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="G18" s="38" t="s">
-        <v>68</v>
-      </c>
-      <c r="H18" s="41">
-        <v>11</v>
-      </c>
-      <c r="I18" s="36">
-        <v>46179</v>
-      </c>
-      <c r="K18" s="37"/>
-      <c r="L18" s="37"/>
-      <c r="M18" s="37"/>
-    </row>
-    <row r="19" ht="37.5">
-      <c r="A19" s="31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="31" t="s">
-        <v>71</v>
-      </c>
-      <c r="C19" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="D19" s="31" t="s">
+      <c r="G19" s="38" t="s">
         <v>73</v>
       </c>
-      <c r="E19" s="34" t="s">
-        <v>64</v>
-      </c>
-      <c r="F19" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G19" s="42" t="s">
-        <v>74</v>
-      </c>
-      <c r="H19" s="32">
+      <c r="H19" s="37">
         <v>12</v>
       </c>
-      <c r="I19" s="36"/>
-      <c r="K19" s="37"/>
-      <c r="L19" s="37"/>
-      <c r="M19" s="37"/>
+      <c r="I19" s="32"/>
+      <c r="K19" s="33"/>
+      <c r="L19" s="33"/>
+      <c r="M19" s="33"/>
     </row>
     <row r="20" ht="19.5" customHeight="1">
       <c r="A20" s="28"/>
@@ -3154,163 +3128,163 @@
       <c r="C20" s="28"/>
       <c r="D20" s="20"/>
       <c r="E20" s="20"/>
-      <c r="F20" s="43"/>
+      <c r="F20" s="39"/>
       <c r="G20" s="20"/>
       <c r="H20" s="20"/>
       <c r="I20" s="25"/>
-      <c r="K20" s="37"/>
-      <c r="L20" s="37"/>
-      <c r="M20" s="37"/>
+      <c r="K20" s="33"/>
+      <c r="L20" s="33"/>
+      <c r="M20" s="33"/>
     </row>
     <row r="21" ht="19.5" customHeight="1">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="C21" s="40" t="s">
         <v>76</v>
       </c>
-      <c r="C21" s="44" t="s">
+      <c r="D21" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="D21" s="44" t="s">
+      <c r="E21" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="E21" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G21" s="31" t="s">
+      <c r="H21" s="11">
+        <v>11</v>
+      </c>
+      <c r="I21" s="18"/>
+      <c r="K21" s="33"/>
+      <c r="L21" s="33"/>
+      <c r="M21" s="33"/>
+    </row>
+    <row r="22" ht="19.5" customHeight="1">
+      <c r="A22" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="H21" s="32">
+      <c r="C22" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H22" s="11">
         <v>11</v>
       </c>
-      <c r="I21" s="18"/>
-      <c r="K21" s="37"/>
-      <c r="L21" s="37"/>
-      <c r="M21" s="37"/>
-    </row>
-    <row r="22" ht="19.5" customHeight="1">
-      <c r="A22" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="B22" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="C22" s="44" t="s">
-        <v>81</v>
-      </c>
-      <c r="D22" s="44" t="s">
+      <c r="I22" s="18"/>
+      <c r="K22" s="33"/>
+      <c r="L22" s="33"/>
+      <c r="M22" s="33"/>
+    </row>
+    <row r="23" ht="19.5" customHeight="1">
+      <c r="A23" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="E22" s="45" t="s">
+      <c r="C23" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D23" s="40" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G22" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H22" s="32">
+      <c r="F23" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H23" s="11">
         <v>11</v>
       </c>
-      <c r="I22" s="18"/>
-      <c r="K22" s="37"/>
-      <c r="L22" s="37"/>
-      <c r="M22" s="37"/>
-    </row>
-    <row r="23" ht="19.5" customHeight="1">
-      <c r="A23" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="C23" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="D23" s="44" t="s">
+      <c r="I23" s="18"/>
+      <c r="K23" s="33"/>
+      <c r="L23" s="33"/>
+      <c r="M23" s="33"/>
+    </row>
+    <row r="24" ht="19.5" customHeight="1">
+      <c r="A24" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E23" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G23" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H23" s="32">
+      <c r="C24" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="D24" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H24" s="11">
         <v>11</v>
       </c>
-      <c r="I23" s="18"/>
-      <c r="K23" s="37"/>
-      <c r="L23" s="37"/>
-      <c r="M23" s="37"/>
-    </row>
-    <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" s="31" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="44" t="s">
-        <v>87</v>
-      </c>
-      <c r="D24" s="44" t="s">
+      <c r="I24" s="18"/>
+      <c r="K24" s="33"/>
+      <c r="L24" s="33"/>
+      <c r="M24" s="33"/>
+    </row>
+    <row r="25" ht="19.5" customHeight="1">
+      <c r="A25" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="E24" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="F24" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G24" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H24" s="32">
+      <c r="C25" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="H25" s="11">
         <v>11</v>
       </c>
-      <c r="I24" s="18"/>
-      <c r="K24" s="37"/>
-      <c r="L24" s="37"/>
-      <c r="M24" s="37"/>
-    </row>
-    <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="D25" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="E25" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="F25" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G25" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H25" s="32">
-        <v>11</v>
-      </c>
       <c r="I25" s="18"/>
-      <c r="K25" s="37"/>
-      <c r="L25" s="37"/>
-      <c r="M25" s="37"/>
+      <c r="K25" s="33"/>
+      <c r="L25" s="33"/>
+      <c r="M25" s="33"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
       <c r="A26" s="28"/>
@@ -3318,133 +3292,133 @@
       <c r="C26" s="28"/>
       <c r="D26" s="28"/>
       <c r="E26" s="20"/>
-      <c r="F26" s="43"/>
+      <c r="F26" s="39"/>
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
       <c r="I26" s="25"/>
-      <c r="K26" s="37"/>
-      <c r="L26" s="37"/>
-      <c r="M26" s="37"/>
+      <c r="K26" s="33"/>
+      <c r="L26" s="33"/>
+      <c r="M26" s="33"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="31" t="s">
+      <c r="A27" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B27" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="C27" s="40" t="s">
         <v>94</v>
       </c>
-      <c r="C27" s="44" t="s">
+      <c r="D27" s="40" t="s">
         <v>95</v>
       </c>
-      <c r="D27" s="44" t="s">
+      <c r="E27" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="E27" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G27" s="31" t="s">
+      <c r="H27" s="11">
+        <v>8</v>
+      </c>
+      <c r="I27" s="18"/>
+      <c r="K27" s="33"/>
+      <c r="L27" s="33"/>
+      <c r="M27" s="33"/>
+    </row>
+    <row r="28" ht="19.5" customHeight="1">
+      <c r="A28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="H27" s="32">
+      <c r="C28" s="40" t="s">
+        <v>98</v>
+      </c>
+      <c r="D28" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="E28" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H28" s="11">
+        <v>10</v>
+      </c>
+      <c r="I28" s="18"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="33"/>
+      <c r="M28" s="33"/>
+    </row>
+    <row r="29" ht="19.5" customHeight="1">
+      <c r="A29" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" s="40" t="s">
+        <v>102</v>
+      </c>
+      <c r="E29" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H29" s="11">
         <v>8</v>
       </c>
-      <c r="I27" s="18"/>
-      <c r="K27" s="37"/>
-      <c r="L27" s="37"/>
-      <c r="M27" s="37"/>
-    </row>
-    <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="B28" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="44" t="s">
-        <v>99</v>
-      </c>
-      <c r="D28" s="44" t="s">
-        <v>100</v>
-      </c>
-      <c r="E28" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F28" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G28" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="H28" s="32">
-        <v>10</v>
-      </c>
-      <c r="I28" s="18"/>
-      <c r="K28" s="37"/>
-      <c r="L28" s="37"/>
-      <c r="M28" s="37"/>
-    </row>
-    <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="B29" s="31" t="s">
-        <v>101</v>
-      </c>
-      <c r="C29" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="D29" s="44" t="s">
+      <c r="I29" s="18"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+    </row>
+    <row r="30" ht="19.5" customHeight="1">
+      <c r="A30" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="E29" s="32" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G29" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="H29" s="32">
+      <c r="C30" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="D30" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="E30" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="H30" s="11">
         <v>8</v>
       </c>
-      <c r="I29" s="18"/>
-      <c r="K29" s="37"/>
-      <c r="L29" s="37"/>
-      <c r="M29" s="37"/>
-    </row>
-    <row r="30" ht="19.5" customHeight="1">
-      <c r="A30" s="31" t="s">
-        <v>93</v>
-      </c>
-      <c r="B30" s="31" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="44" t="s">
-        <v>105</v>
-      </c>
-      <c r="D30" s="44" t="s">
-        <v>106</v>
-      </c>
-      <c r="E30" s="32" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G30" s="31" t="s">
-        <v>97</v>
-      </c>
-      <c r="H30" s="32">
-        <v>8</v>
-      </c>
       <c r="I30" s="18"/>
-      <c r="K30" s="37"/>
-      <c r="L30" s="37"/>
-      <c r="M30" s="37"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" s="28"/>
@@ -3452,7 +3426,7 @@
       <c r="C31" s="28"/>
       <c r="D31" s="20"/>
       <c r="E31" s="20"/>
-      <c r="F31" s="43"/>
+      <c r="F31" s="39"/>
       <c r="G31" s="20"/>
       <c r="H31" s="20"/>
       <c r="I31" s="25"/>
@@ -3461,98 +3435,98 @@
       <c r="M31" s="1"/>
     </row>
     <row r="32" ht="19.5" customHeight="1">
-      <c r="A32" s="31" t="s">
+      <c r="A32" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B32" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="C32" s="40" t="s">
         <v>108</v>
       </c>
-      <c r="C32" s="44" t="s">
+      <c r="D32" s="40" t="s">
         <v>109</v>
       </c>
-      <c r="D32" s="44" t="s">
+      <c r="E32" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E32" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G32" s="31" t="s">
+      <c r="H32" s="11">
+        <v>7</v>
+      </c>
+      <c r="I32" s="18"/>
+    </row>
+    <row r="33" ht="19.5" customHeight="1">
+      <c r="A33" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="H32" s="32">
+      <c r="C33" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="D33" s="40" t="s">
+        <v>113</v>
+      </c>
+      <c r="E33" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H33" s="11">
         <v>7</v>
       </c>
-      <c r="I32" s="18"/>
-    </row>
-    <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="B33" s="31" t="s">
-        <v>112</v>
-      </c>
-      <c r="C33" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="D33" s="44" t="s">
+      <c r="I33" s="18"/>
+    </row>
+    <row r="34" ht="19.5" customHeight="1">
+      <c r="A34" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="E33" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F33" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G33" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="H33" s="32">
-        <v>7</v>
-      </c>
-      <c r="I33" s="18"/>
-    </row>
-    <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="B34" s="31" t="s">
+      <c r="C34" s="40" t="s">
         <v>115</v>
       </c>
-      <c r="C34" s="44" t="s">
+      <c r="D34" s="40" t="s">
         <v>116</v>
       </c>
-      <c r="D34" s="44" t="s">
-        <v>117</v>
-      </c>
-      <c r="E34" s="32" t="s">
+      <c r="E34" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="F34" s="35" t="s">
-        <v>50</v>
-      </c>
-      <c r="G34" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="H34" s="32">
+      <c r="F34" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="H34" s="11">
         <v>7</v>
       </c>
       <c r="I34" s="18"/>
     </row>
     <row r="35" ht="19.5" customHeight="1">
       <c r="A35" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B35" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="C35" s="40" t="s">
         <v>118</v>
       </c>
-      <c r="C35" s="46" t="s">
+      <c r="D35" s="40" t="s">
         <v>119</v>
-      </c>
-      <c r="D35" s="46" t="s">
-        <v>120</v>
       </c>
       <c r="E35" s="11" t="s">
         <v>33</v>
@@ -3561,7 +3535,7 @@
         <v>14</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H35" s="11">
         <v>6</v>
@@ -3570,25 +3544,25 @@
     </row>
     <row r="36" ht="19.5" customHeight="1">
       <c r="A36" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C36" s="40" t="s">
         <v>121</v>
       </c>
-      <c r="C36" s="46" t="s">
+      <c r="D36" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="D36" s="46" t="s">
-        <v>123</v>
-      </c>
       <c r="E36" s="11" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>14</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H36" s="11">
         <v>7</v>
@@ -3601,32 +3575,32 @@
       <c r="C37" s="28"/>
       <c r="D37" s="20"/>
       <c r="E37" s="20"/>
-      <c r="F37" s="43"/>
+      <c r="F37" s="39"/>
       <c r="G37" s="20"/>
       <c r="H37" s="20"/>
       <c r="I37" s="25"/>
     </row>
     <row r="38" ht="19.5" customHeight="1">
       <c r="A38" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="C38" s="40" t="s">
         <v>125</v>
       </c>
-      <c r="C38" s="46" t="s">
+      <c r="D38" s="40" t="s">
         <v>126</v>
       </c>
-      <c r="D38" s="46" t="s">
-        <v>127</v>
-      </c>
-      <c r="E38" s="47" t="s">
+      <c r="E38" s="41" t="s">
         <v>26</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>14</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H38" s="11">
         <v>10</v>
@@ -3635,25 +3609,25 @@
     </row>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B39" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C39" s="40" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="46" t="s">
+      <c r="D39" s="40" t="s">
         <v>130</v>
       </c>
-      <c r="D39" s="46" t="s">
+      <c r="E39" s="11" t="s">
         <v>131</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>132</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>14</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H39" s="11">
         <v>11</v>
@@ -3661,16 +3635,16 @@
       <c r="I39" s="18"/>
     </row>
     <row r="40" ht="19.5" customHeight="1">
-      <c r="A40" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="B40" s="48"/>
-      <c r="C40" s="48"/>
-      <c r="D40" s="48"/>
-      <c r="E40" s="48"/>
-      <c r="F40" s="48"/>
-      <c r="G40" s="48"/>
-      <c r="H40" s="49">
+      <c r="A40" s="42" t="s">
+        <v>132</v>
+      </c>
+      <c r="B40" s="42"/>
+      <c r="C40" s="42"/>
+      <c r="D40" s="42"/>
+      <c r="E40" s="42"/>
+      <c r="F40" s="42"/>
+      <c r="G40" s="42"/>
+      <c r="H40" s="43">
         <f>SUM(H2,H3,H4,H5,H6,H8,H9,H10,H12,H13,H15,H17,H18,H21,H22,H23,H24,H25,H27,H28,H29,H30,H32,H33,H34,H35,H36,H38,H39)</f>
         <v>331</v>
       </c>
@@ -3679,236 +3653,236 @@
       <c r="A41" s="1"/>
     </row>
     <row r="42" ht="17.25">
-      <c r="A42" s="50"/>
-      <c r="B42" s="51"/>
-      <c r="C42" s="51"/>
-      <c r="F42" s="52"/>
+      <c r="A42" s="44"/>
+      <c r="B42" s="44"/>
+      <c r="C42" s="44"/>
+      <c r="F42" s="45"/>
     </row>
     <row r="43" ht="17.25">
-      <c r="A43" s="50"/>
-      <c r="B43" s="51"/>
-      <c r="C43" s="51"/>
-      <c r="F43" s="52"/>
+      <c r="A43" s="44"/>
+      <c r="B43" s="44"/>
+      <c r="C43" s="44"/>
+      <c r="F43" s="45"/>
     </row>
     <row r="44" ht="17.25">
-      <c r="A44" s="50"/>
-      <c r="B44" s="51"/>
-      <c r="C44" s="51"/>
-      <c r="F44" s="52"/>
+      <c r="A44" s="44"/>
+      <c r="B44" s="44"/>
+      <c r="C44" s="44"/>
+      <c r="F44" s="45"/>
     </row>
     <row r="45" ht="17.25">
-      <c r="A45" s="50"/>
-      <c r="B45" s="51"/>
-      <c r="C45" s="51"/>
-      <c r="F45" s="52"/>
+      <c r="A45" s="44"/>
+      <c r="B45" s="44"/>
+      <c r="C45" s="44"/>
+      <c r="F45" s="45"/>
     </row>
     <row r="46" ht="17.25">
       <c r="A46" s="1"/>
-      <c r="F46" s="52"/>
+      <c r="F46" s="45"/>
     </row>
     <row r="47" ht="17.25">
-      <c r="A47" s="50"/>
-      <c r="B47" s="50"/>
-      <c r="C47" s="50"/>
-      <c r="D47" s="50"/>
-      <c r="F47" s="52"/>
+      <c r="A47" s="44"/>
+      <c r="B47" s="44"/>
+      <c r="C47" s="44"/>
+      <c r="D47" s="44"/>
+      <c r="F47" s="45"/>
     </row>
     <row r="48" ht="17.25">
-      <c r="A48" s="50"/>
-      <c r="B48" s="51"/>
-      <c r="C48" s="51"/>
-      <c r="F48" s="52"/>
-      <c r="K48" s="53"/>
+      <c r="A48" s="44"/>
+      <c r="B48" s="44"/>
+      <c r="C48" s="44"/>
+      <c r="F48" s="45"/>
+      <c r="K48" s="46"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
     </row>
     <row r="49" ht="17.25">
-      <c r="A49" s="50"/>
-      <c r="B49" s="51"/>
-      <c r="C49" s="51"/>
-      <c r="F49" s="52"/>
+      <c r="A49" s="44"/>
+      <c r="B49" s="44"/>
+      <c r="C49" s="44"/>
+      <c r="F49" s="45"/>
     </row>
     <row r="50" ht="17.25">
-      <c r="A50" s="50"/>
-      <c r="B50" s="51"/>
-      <c r="C50" s="51"/>
-      <c r="F50" s="52"/>
+      <c r="A50" s="44"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="44"/>
+      <c r="F50" s="45"/>
     </row>
     <row r="51" ht="17.25">
-      <c r="A51" s="50"/>
-      <c r="B51" s="51"/>
-      <c r="C51" s="51"/>
-      <c r="F51" s="52"/>
+      <c r="A51" s="44"/>
+      <c r="B51" s="44"/>
+      <c r="C51" s="44"/>
+      <c r="F51" s="45"/>
     </row>
     <row r="52" ht="17.25">
-      <c r="A52" s="50"/>
-      <c r="B52" s="51"/>
-      <c r="C52" s="51"/>
-      <c r="F52" s="52"/>
+      <c r="A52" s="44"/>
+      <c r="B52" s="44"/>
+      <c r="C52" s="44"/>
+      <c r="F52" s="45"/>
     </row>
     <row r="53" ht="17.25">
-      <c r="A53" s="50"/>
-      <c r="B53" s="51"/>
-      <c r="C53" s="51"/>
-      <c r="F53" s="52"/>
+      <c r="A53" s="44"/>
+      <c r="B53" s="44"/>
+      <c r="C53" s="44"/>
+      <c r="F53" s="45"/>
     </row>
     <row r="54" ht="17.25">
       <c r="A54" s="1"/>
-      <c r="F54" s="52"/>
+      <c r="F54" s="45"/>
     </row>
     <row r="55" ht="17.25">
-      <c r="A55" s="50"/>
-      <c r="B55" s="50"/>
-      <c r="C55" s="50"/>
-      <c r="D55" s="50"/>
-      <c r="F55" s="52"/>
+      <c r="A55" s="44"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
+      <c r="D55" s="44"/>
+      <c r="F55" s="45"/>
     </row>
     <row r="56" ht="17.25">
-      <c r="A56" s="50"/>
-      <c r="B56" s="51"/>
-      <c r="C56" s="51"/>
-      <c r="F56" s="52"/>
+      <c r="A56" s="44"/>
+      <c r="B56" s="44"/>
+      <c r="C56" s="44"/>
+      <c r="F56" s="45"/>
     </row>
     <row r="57" ht="17.25">
-      <c r="A57" s="50"/>
-      <c r="B57" s="51"/>
-      <c r="C57" s="51"/>
-      <c r="F57" s="52"/>
+      <c r="A57" s="44"/>
+      <c r="B57" s="44"/>
+      <c r="C57" s="44"/>
+      <c r="F57" s="45"/>
     </row>
     <row r="58" ht="17.25">
-      <c r="A58" s="50"/>
-      <c r="B58" s="51"/>
-      <c r="C58" s="51"/>
-      <c r="F58" s="52"/>
+      <c r="A58" s="44"/>
+      <c r="B58" s="44"/>
+      <c r="C58" s="44"/>
+      <c r="F58" s="45"/>
     </row>
     <row r="59" ht="18.75">
-      <c r="A59" s="50"/>
-      <c r="B59" s="50"/>
-      <c r="C59" s="50"/>
+      <c r="A59" s="44"/>
+      <c r="B59" s="44"/>
+      <c r="C59" s="44"/>
       <c r="D59" s="1"/>
-      <c r="F59" s="52"/>
+      <c r="F59" s="45"/>
     </row>
     <row r="60" ht="18.75">
       <c r="A60" s="1"/>
-      <c r="B60" s="54"/>
-      <c r="C60" s="54"/>
-      <c r="F60" s="52"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="F60" s="45"/>
     </row>
     <row r="61" ht="17.25">
-      <c r="A61" s="50"/>
-      <c r="B61" s="50"/>
-      <c r="C61" s="50"/>
-      <c r="D61" s="50"/>
-      <c r="F61" s="52"/>
+      <c r="A61" s="44"/>
+      <c r="B61" s="44"/>
+      <c r="C61" s="44"/>
+      <c r="D61" s="44"/>
+      <c r="F61" s="45"/>
     </row>
     <row r="62" ht="17.25">
-      <c r="A62" s="50"/>
-      <c r="B62" s="51"/>
-      <c r="C62" s="51"/>
-      <c r="F62" s="52"/>
+      <c r="A62" s="44"/>
+      <c r="B62" s="44"/>
+      <c r="C62" s="44"/>
+      <c r="F62" s="45"/>
     </row>
     <row r="63" ht="17.25">
-      <c r="A63" s="50"/>
-      <c r="B63" s="51"/>
-      <c r="C63" s="51"/>
-      <c r="F63" s="52"/>
+      <c r="A63" s="44"/>
+      <c r="B63" s="44"/>
+      <c r="C63" s="44"/>
+      <c r="F63" s="45"/>
     </row>
     <row r="64" ht="17.25">
-      <c r="A64" s="50"/>
-      <c r="B64" s="51"/>
-      <c r="C64" s="51"/>
-      <c r="F64" s="52"/>
+      <c r="A64" s="44"/>
+      <c r="B64" s="44"/>
+      <c r="C64" s="44"/>
+      <c r="F64" s="45"/>
     </row>
     <row r="65" ht="17.25">
-      <c r="A65" s="50"/>
-      <c r="B65" s="51"/>
-      <c r="C65" s="51"/>
-      <c r="F65" s="52"/>
+      <c r="A65" s="44"/>
+      <c r="B65" s="44"/>
+      <c r="C65" s="44"/>
+      <c r="F65" s="45"/>
     </row>
     <row r="66" ht="14.25">
-      <c r="A66" s="50"/>
-      <c r="B66" s="51"/>
-      <c r="C66" s="51"/>
-      <c r="F66" s="52"/>
+      <c r="A66" s="44"/>
+      <c r="B66" s="44"/>
+      <c r="C66" s="44"/>
+      <c r="F66" s="45"/>
     </row>
     <row r="67" ht="14.25">
       <c r="A67" s="1"/>
-      <c r="F67" s="52"/>
+      <c r="F67" s="45"/>
     </row>
     <row r="68" ht="14.25">
-      <c r="A68" s="50"/>
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
-      <c r="D68" s="50"/>
-      <c r="F68" s="52"/>
+      <c r="A68" s="44"/>
+      <c r="B68" s="44"/>
+      <c r="C68" s="44"/>
+      <c r="D68" s="44"/>
+      <c r="F68" s="45"/>
     </row>
     <row r="69" ht="14.25">
-      <c r="A69" s="50"/>
-      <c r="B69" s="51"/>
-      <c r="C69" s="51"/>
-      <c r="F69" s="52"/>
+      <c r="A69" s="44"/>
+      <c r="B69" s="44"/>
+      <c r="C69" s="44"/>
+      <c r="F69" s="45"/>
     </row>
     <row r="70" ht="14.25">
-      <c r="A70" s="50"/>
-      <c r="B70" s="51"/>
-      <c r="C70" s="51"/>
-      <c r="F70" s="52"/>
+      <c r="A70" s="44"/>
+      <c r="B70" s="44"/>
+      <c r="C70" s="44"/>
+      <c r="F70" s="45"/>
     </row>
     <row r="71" ht="14.25">
-      <c r="A71" s="50"/>
-      <c r="B71" s="50"/>
-      <c r="C71" s="50"/>
+      <c r="A71" s="44"/>
+      <c r="B71" s="44"/>
+      <c r="C71" s="44"/>
       <c r="D71" s="1"/>
-      <c r="F71" s="52"/>
+      <c r="F71" s="45"/>
     </row>
     <row r="72" ht="14.25">
-      <c r="A72" s="50"/>
-      <c r="B72" s="51"/>
-      <c r="C72" s="51"/>
-      <c r="F72" s="52"/>
+      <c r="A72" s="44"/>
+      <c r="B72" s="44"/>
+      <c r="C72" s="44"/>
+      <c r="F72" s="45"/>
     </row>
     <row r="73" ht="14.25">
-      <c r="A73" s="50"/>
-      <c r="B73" s="51"/>
-      <c r="C73" s="51"/>
-      <c r="F73" s="52"/>
+      <c r="A73" s="44"/>
+      <c r="B73" s="44"/>
+      <c r="C73" s="44"/>
+      <c r="F73" s="45"/>
     </row>
     <row r="74" ht="14.25">
       <c r="A74" s="1"/>
-      <c r="B74" s="54"/>
-      <c r="C74" s="54"/>
-      <c r="F74" s="52"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="F74" s="45"/>
     </row>
     <row r="75" ht="14.25">
-      <c r="A75" s="50"/>
-      <c r="B75" s="50"/>
-      <c r="C75" s="50"/>
-      <c r="D75" s="50"/>
-      <c r="F75" s="52"/>
+      <c r="A75" s="44"/>
+      <c r="B75" s="44"/>
+      <c r="C75" s="44"/>
+      <c r="D75" s="44"/>
+      <c r="F75" s="45"/>
     </row>
     <row r="76" ht="14.25">
-      <c r="A76" s="50"/>
-      <c r="B76" s="51"/>
-      <c r="C76" s="51"/>
-      <c r="F76" s="52"/>
+      <c r="A76" s="44"/>
+      <c r="B76" s="44"/>
+      <c r="C76" s="44"/>
+      <c r="F76" s="45"/>
     </row>
     <row r="77" ht="14.25">
-      <c r="A77" s="50"/>
-      <c r="B77" s="51"/>
-      <c r="C77" s="51"/>
-      <c r="F77" s="52"/>
+      <c r="A77" s="44"/>
+      <c r="B77" s="44"/>
+      <c r="C77" s="44"/>
+      <c r="F77" s="45"/>
     </row>
     <row r="78" ht="14.25">
-      <c r="A78" s="50"/>
-      <c r="B78" s="51"/>
-      <c r="C78" s="51"/>
-      <c r="F78" s="52"/>
+      <c r="A78" s="44"/>
+      <c r="B78" s="44"/>
+      <c r="C78" s="44"/>
+      <c r="F78" s="45"/>
     </row>
     <row r="79" ht="14.25">
-      <c r="A79" s="50"/>
-      <c r="B79" s="51"/>
-      <c r="C79" s="51"/>
-      <c r="F79" s="52"/>
+      <c r="A79" s="44"/>
+      <c r="B79" s="44"/>
+      <c r="C79" s="44"/>
+      <c r="F79" s="45"/>
     </row>
     <row r="80" ht="14.25">
       <c r="A80" s="1"/>
@@ -3922,28 +3896,28 @@
     </row>
     <row r="83" ht="14.25">
       <c r="A83" s="1"/>
-      <c r="B83" s="54"/>
-      <c r="C83" s="54"/>
+      <c r="B83" s="1"/>
+      <c r="C83" s="1"/>
     </row>
     <row r="84" ht="14.25">
       <c r="A84" s="1"/>
-      <c r="B84" s="54"/>
-      <c r="C84" s="54"/>
+      <c r="B84" s="1"/>
+      <c r="C84" s="1"/>
     </row>
     <row r="85" ht="14.25">
       <c r="A85" s="1"/>
-      <c r="B85" s="54"/>
-      <c r="C85" s="54"/>
+      <c r="B85" s="1"/>
+      <c r="C85" s="1"/>
     </row>
     <row r="86" ht="14.25">
       <c r="A86" s="1"/>
-      <c r="B86" s="54"/>
-      <c r="C86" s="54"/>
+      <c r="B86" s="1"/>
+      <c r="C86" s="1"/>
     </row>
     <row r="87" ht="14.25">
       <c r="A87" s="1"/>
-      <c r="B87" s="54"/>
-      <c r="C87" s="54"/>
+      <c r="B87" s="1"/>
+      <c r="C87" s="1"/>
     </row>
     <row r="88" ht="14.25">
       <c r="A88" s="1"/>
@@ -3959,23 +3933,23 @@
     </row>
     <row r="93" ht="14.25">
       <c r="A93" s="1"/>
-      <c r="B93" s="54"/>
-      <c r="C93" s="54"/>
+      <c r="B93" s="1"/>
+      <c r="C93" s="1"/>
     </row>
     <row r="94" ht="14.25">
       <c r="A94" s="1"/>
-      <c r="B94" s="54"/>
-      <c r="C94" s="54"/>
+      <c r="B94" s="1"/>
+      <c r="C94" s="1"/>
     </row>
     <row r="95" ht="14.25">
       <c r="A95" s="1"/>
-      <c r="B95" s="54"/>
-      <c r="C95" s="54"/>
+      <c r="B95" s="1"/>
+      <c r="C95" s="1"/>
     </row>
     <row r="96" ht="14.25">
       <c r="A96" s="1"/>
-      <c r="B96" s="54"/>
-      <c r="C96" s="54"/>
+      <c r="B96" s="1"/>
+      <c r="C96" s="1"/>
     </row>
     <row r="97" ht="14.25">
       <c r="A97" s="1"/>

</xml_diff>